<commit_message>
Major update: refactor pipeline and project structure
</commit_message>
<xml_diff>
--- a/stage_6_results_analysis/output/final_review_summary.xlsx
+++ b/stage_6_results_analysis/output/final_review_summary.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,112 +457,112 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Records imported</t>
+          <t>Records received for abstract screening</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1170</v>
+        <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/input/abstract_screening_input.xlsx</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Records after merge</t>
+          <t>Records received for full-text screening</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1170</v>
+        <v>0</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/input/fulltext_screening_input.xlsx</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 4</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Exact duplicate groups identified</t>
+          <t>Paper-level pairing records</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>202</v>
+        <v>0</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/paper_level_framework_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Exact duplicates removed</t>
+          <t>Pair-level CT-programming records</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Records retained after exact deduplication</t>
+          <t>Characterized papers</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>935</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_5_characterization/output/results_characterization.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Possible fuzzy duplicates for manual review</t>
+          <t>Framework-following papers with at least one CT-programming pair</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -570,465 +570,125 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Records excluded before title screening as non-screenable</t>
+          <t>Total CT-programming pair records following the framework</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Records screened by title</t>
+          <t>Unique CT-programming pair types following the framework</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>876</v>
+        <v>0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Title screening Yes</t>
+          <t>Mapped papers in paper-level dataset</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>215</v>
+        <v>84</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>Stage 6 runtime</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 6</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Title screening Partially</t>
+          <t>Characterization papers loaded</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>479</v>
+        <v>84</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>Stage 6 runtime</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 6</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Title screening No</t>
+          <t>Papers kept for final analysis</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>182</v>
+        <v>84</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+          <t>Stage 6 runtime</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Stage 1</t>
+          <t>Stage 6</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Title screening Undetermined</t>
+          <t>Mapped Paper_IDs missing from characterization dataset</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Stage 1</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Records sent to abstract screening</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>694</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Stage 1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Poster/demo/WIP/extended abstract candidates sent to title screening</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>17</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Stage 1</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Missing abstracts sent to title screening</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>37</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Stage 1</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Short abstracts sent to title screening</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>18</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Stage 1</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Possibly truncated abstracts sent to title screening</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>4</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Stage 2</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Records received for abstract screening</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>694</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/input/abstract_screening_input.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Stage 3</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Records received for full-text screening</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>301</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/input/fulltext_screening_input.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Stage 4</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Paper-level pairing records</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>84</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/paper_level_framework_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Stage 4</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Pair-level CT-programming records</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>185</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Stage 5</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Characterized papers</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>84</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_5_characterization/output/results_characterization.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Stage 4</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Framework-following papers with at least one CT-programming pair</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>60</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Stage 4</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Total CT-programming pair records following the framework</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>185</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Stage 4</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Unique CT-programming pair types following the framework</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>44</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Stage 6</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Mapped papers in paper-level dataset</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>84</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Stage 6 runtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Stage 6</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Characterization papers loaded</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>84</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Stage 6 runtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Stage 6</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Papers kept for final analysis</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>84</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Stage 6 runtime</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Stage 6</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Mapped Paper_IDs missing from characterization dataset</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" t="inlineStr">
         <is>
           <t>Stage 6 runtime</t>
         </is>
@@ -1100,7 +760,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/output/abstracts_screened_llm_llm_costs.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/output/stage_2_costs.xlsx</t>
         </is>
       </c>
     </row>
@@ -1124,7 +784,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/output/fulltext_llm_costs.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/output/stage_3_costs.xlsx</t>
         </is>
       </c>
     </row>
@@ -1172,7 +832,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_5_characterization/output/characterization_llm_costs.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_5_characterization/output/stage_5_llm_costs.xlsx</t>
         </is>
       </c>
     </row>
@@ -1239,7 +899,7 @@
         </is>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1254,7 +914,7 @@
         </is>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1265,7 +925,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/output/abstracts_screened_llm_results.xlsx</t>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/output/stage_2_results.xlsx</t>
         </is>
       </c>
       <c r="C4" t="b">
@@ -1284,7 +944,7 @@
         </is>
       </c>
       <c r="C5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1299,7 +959,7 @@
         </is>
       </c>
       <c r="C6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1314,7 +974,7 @@
         </is>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1329,7 +989,7 @@
         </is>
       </c>
       <c r="C8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1344,7 +1004,7 @@
         </is>
       </c>
       <c r="C9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1358,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1376,6 +1036,111 @@
         <is>
           <t>Exists</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Stage 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_1_import_filtering/output/review_pipeline_processing.xlsx</t>
+        </is>
+      </c>
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_2_abstract_screening/input/abstract_screening_input.xlsx</t>
+        </is>
+      </c>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/input/fulltext_screening_input.xlsx</t>
+        </is>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Stage 3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_3_fulltext_initial_pairing/output/fulltext_results.xlsx</t>
+        </is>
+      </c>
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Stage 4</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/paper_level_framework_results.xlsx</t>
+        </is>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Stage 4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_4_full_pairing/output/pair_level_mapping_results.xlsx</t>
+        </is>
+      </c>
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Stage 5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>/home/tania/llm_project_env/Scoping_Review_CTProgra/stage_5_characterization/output/results_characterization.xlsx</t>
+        </is>
+      </c>
+      <c r="C8" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>